<commit_message>
add country variable to coded articles
</commit_message>
<xml_diff>
--- a/outputs/coding-answers-human/testList_answers_df_v9_human.xlsx
+++ b/outputs/coding-answers-human/testList_answers_df_v9_human.xlsx
@@ -14,12 +14,15 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AQ$25</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="580">
   <si>
     <t>id</t>
   </si>
@@ -3836,6 +3839,54 @@
   </si>
   <si>
     <t>['Interview', 'Workshop']</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>['Norway']</t>
+  </si>
+  <si>
+    <t>['India']</t>
+  </si>
+  <si>
+    <t>['United States']</t>
+  </si>
+  <si>
+    <t>['Peru']</t>
+  </si>
+  <si>
+    <t>['Thailand', 'Philippines']</t>
+  </si>
+  <si>
+    <t>['South Africa']</t>
+  </si>
+  <si>
+    <t>['Philippines']</t>
+  </si>
+  <si>
+    <t>['The Gambia']</t>
+  </si>
+  <si>
+    <t>['Solomon Islands']</t>
+  </si>
+  <si>
+    <t>['Australia']</t>
+  </si>
+  <si>
+    <t>['Bangladesh']</t>
+  </si>
+  <si>
+    <t>['Senegal']</t>
+  </si>
+  <si>
+    <t>['Japan']</t>
+  </si>
+  <si>
+    <t>['Trinidad and Tobago']</t>
+  </si>
+  <si>
+    <t>['Asia', 'Africa', 'Oceania']</t>
   </si>
 </sst>
 </file>
@@ -4241,7 +4292,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AP25"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:AQ25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8.7265625" style="3"/>
@@ -4250,14 +4302,14 @@
     <col min="13" max="13" width="8.7265625" style="3"/>
     <col min="17" max="17" width="8.7265625" style="3"/>
     <col min="20" max="20" width="8.7265625" style="3"/>
-    <col min="23" max="24" width="8.7265625" style="3"/>
-    <col min="28" max="28" width="8.7265625" style="3"/>
-    <col min="29" max="29" width="8.7265625" style="8"/>
-    <col min="33" max="33" width="8.7265625" style="3"/>
-    <col min="36" max="37" width="8.7265625" style="3"/>
+    <col min="23" max="25" width="8.7265625" style="3"/>
+    <col min="29" max="29" width="8.7265625" style="3"/>
+    <col min="30" max="30" width="8.7265625" style="8"/>
+    <col min="34" max="34" width="8.7265625" style="3"/>
+    <col min="37" max="38" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4330,62 +4382,65 @@
       <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="7" t="s">
+      <c r="AD1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AH1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="11" t="s">
+      <c r="AP1" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>71</v>
       </c>
@@ -4413,26 +4468,29 @@
       <c r="X2" s="3" t="s">
         <v>527</v>
       </c>
-      <c r="AB2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="AC2" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="AC2" s="8" t="s">
+      <c r="AD2" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AG2" s="3" t="b">
+      <c r="AH2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AJ2" s="3" t="s">
+      <c r="AK2" s="3" t="s">
         <v>528</v>
       </c>
-      <c r="AK2" s="3" t="s">
+      <c r="AL2" s="3" t="s">
         <v>529</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AP2" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>85</v>
       </c>
@@ -4494,50 +4552,53 @@
         <v>57</v>
       </c>
       <c r="X3" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>332</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>333</v>
+      </c>
+      <c r="AC3" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="AD3" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>334</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>138</v>
+      </c>
+      <c r="AH3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>335</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>336</v>
+      </c>
+      <c r="AK3" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="AL3" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Y3" t="s">
-        <v>332</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>333</v>
-      </c>
-      <c r="AB3" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="AC3" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>334</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>138</v>
-      </c>
-      <c r="AG3" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>335</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>336</v>
-      </c>
-      <c r="AJ3" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="AK3" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="AL3" t="s">
+      <c r="AM3" t="s">
         <v>337</v>
       </c>
-      <c r="AN3" t="s">
+      <c r="AO3" t="s">
         <v>338</v>
       </c>
-      <c r="AP3" s="6"/>
+      <c r="AQ3" s="6"/>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:43" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>183</v>
       </c>
@@ -4601,50 +4662,50 @@
       <c r="X4" s="3" t="s">
         <v>416</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
         <v>417</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AB4" t="s">
         <v>418</v>
       </c>
-      <c r="AB4" s="3" t="s">
+      <c r="AC4" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="AC4" s="8" t="s">
+      <c r="AD4" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AE4" t="s">
         <v>419</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AF4" t="s">
         <v>138</v>
       </c>
-      <c r="AG4" s="3" t="b">
+      <c r="AH4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH4" t="s">
+      <c r="AI4" t="s">
         <v>420</v>
       </c>
-      <c r="AI4" t="s">
+      <c r="AJ4" t="s">
         <v>421</v>
       </c>
-      <c r="AJ4" s="3" t="s">
+      <c r="AK4" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AK4" s="3" t="s">
+      <c r="AL4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AL4" t="s">
+      <c r="AM4" t="s">
         <v>422</v>
       </c>
-      <c r="AN4" t="s">
+      <c r="AO4" t="s">
         <v>423</v>
       </c>
-      <c r="AP4" t="s">
+      <c r="AQ4" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="5" spans="1:42" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:43" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10">
         <v>252</v>
       </c>
@@ -4708,47 +4769,50 @@
       <c r="X5" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="Y5" s="6" t="s">
+      <c r="Y5" s="4" t="s">
+        <v>567</v>
+      </c>
+      <c r="Z5" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="AA5" s="6" t="s">
+      <c r="AB5" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="AB5" s="4" t="s">
+      <c r="AC5" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="AC5" s="9" t="s">
+      <c r="AD5" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="AD5" s="6" t="s">
+      <c r="AE5" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="AE5" s="6" t="s">
+      <c r="AF5" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="AG5" s="4" t="b">
+      <c r="AH5" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="AH5" s="6" t="s">
+      <c r="AI5" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="AI5" s="6" t="s">
+      <c r="AJ5" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="AJ5" s="4" t="s">
+      <c r="AK5" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AK5" s="4" t="s">
+      <c r="AL5" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="AL5" s="6" t="s">
+      <c r="AM5" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="AN5" s="6" t="s">
+      <c r="AO5" s="6" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>283</v>
       </c>
@@ -4812,47 +4876,50 @@
       <c r="X6" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Y6" s="3" t="s">
+        <v>568</v>
+      </c>
+      <c r="Z6" t="s">
         <v>224</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AB6" t="s">
         <v>225</v>
       </c>
-      <c r="AB6" s="3" t="s">
+      <c r="AC6" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AC6" s="8" t="s">
+      <c r="AD6" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD6" t="s">
+      <c r="AE6" t="s">
         <v>226</v>
       </c>
-      <c r="AE6" t="s">
+      <c r="AF6" t="s">
         <v>117</v>
       </c>
-      <c r="AG6" s="3" t="b">
+      <c r="AH6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH6" t="s">
+      <c r="AI6" t="s">
         <v>227</v>
       </c>
-      <c r="AI6" t="s">
+      <c r="AJ6" t="s">
         <v>228</v>
       </c>
-      <c r="AJ6" s="3" t="s">
+      <c r="AK6" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AK6" s="3" t="s">
+      <c r="AL6" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AL6" t="s">
+      <c r="AM6" t="s">
         <v>229</v>
       </c>
-      <c r="AN6" t="s">
+      <c r="AO6" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>293</v>
       </c>
@@ -4916,47 +4983,50 @@
       <c r="X7" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="Y7" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="Z7" t="s">
         <v>245</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AB7" t="s">
         <v>246</v>
       </c>
-      <c r="AB7" s="3" t="s">
+      <c r="AC7" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AC7" s="8" t="s">
+      <c r="AD7" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="AD7" t="s">
+      <c r="AE7" t="s">
         <v>248</v>
       </c>
-      <c r="AF7" t="s">
+      <c r="AG7" t="s">
         <v>249</v>
       </c>
-      <c r="AG7" s="3" t="b">
+      <c r="AH7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH7" t="s">
+      <c r="AI7" t="s">
         <v>250</v>
       </c>
-      <c r="AI7" t="s">
+      <c r="AJ7" t="s">
         <v>251</v>
       </c>
-      <c r="AJ7" s="3" t="s">
+      <c r="AK7" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AK7" s="3" t="s">
+      <c r="AL7" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="AL7" t="s">
+      <c r="AM7" t="s">
         <v>252</v>
       </c>
-      <c r="AN7" t="s">
+      <c r="AO7" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="8" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>480</v>
       </c>
@@ -5020,47 +5090,50 @@
       <c r="X8" s="3" t="s">
         <v>474</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="Y8" s="3" t="s">
+        <v>570</v>
+      </c>
+      <c r="Z8" t="s">
         <v>475</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AB8" t="s">
         <v>476</v>
       </c>
-      <c r="AB8" s="3" t="s">
+      <c r="AC8" s="3" t="s">
         <v>543</v>
       </c>
-      <c r="AC8" s="8" t="s">
+      <c r="AD8" s="8" t="s">
         <v>477</v>
       </c>
-      <c r="AD8" t="s">
+      <c r="AE8" t="s">
         <v>478</v>
       </c>
-      <c r="AF8" t="s">
+      <c r="AG8" t="s">
         <v>479</v>
       </c>
-      <c r="AG8" s="3" t="b">
+      <c r="AH8" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AH8" t="s">
+      <c r="AI8" t="s">
         <v>480</v>
       </c>
-      <c r="AI8" t="s">
+      <c r="AJ8" t="s">
         <v>481</v>
       </c>
-      <c r="AJ8" s="3" t="s">
+      <c r="AK8" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AK8" s="3" t="s">
+      <c r="AL8" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="AL8" t="s">
+      <c r="AM8" t="s">
         <v>482</v>
       </c>
-      <c r="AN8" t="s">
+      <c r="AO8" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>538</v>
       </c>
@@ -5124,47 +5197,50 @@
       <c r="X9" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Y9" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="Z9" t="s">
         <v>352</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AB9" t="s">
         <v>353</v>
       </c>
-      <c r="AB9" s="3" t="s">
+      <c r="AC9" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="AC9" s="8" t="s">
+      <c r="AD9" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="AE9" t="s">
         <v>355</v>
       </c>
-      <c r="AF9" t="s">
+      <c r="AG9" t="s">
         <v>356</v>
       </c>
-      <c r="AG9" s="3" t="b">
+      <c r="AH9" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AH9" t="s">
+      <c r="AI9" t="s">
         <v>357</v>
       </c>
-      <c r="AI9" t="s">
+      <c r="AJ9" t="s">
         <v>358</v>
       </c>
-      <c r="AJ9" s="3" t="s">
+      <c r="AK9" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="AK9" s="3" t="s">
+      <c r="AL9" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AL9" t="s">
+      <c r="AM9" t="s">
         <v>360</v>
       </c>
-      <c r="AN9" t="s">
+      <c r="AO9" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="10" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:43" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>1290</v>
       </c>
@@ -5228,50 +5304,50 @@
       <c r="X10" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Y10" t="s">
+      <c r="Z10" t="s">
         <v>89</v>
       </c>
-      <c r="AA10" t="s">
+      <c r="AB10" t="s">
         <v>90</v>
       </c>
-      <c r="AB10" s="3" t="s">
+      <c r="AC10" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AC10" s="8" t="s">
+      <c r="AD10" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="AD10" t="s">
+      <c r="AE10" t="s">
         <v>92</v>
       </c>
-      <c r="AF10" t="s">
+      <c r="AG10" t="s">
         <v>93</v>
       </c>
-      <c r="AG10" s="3" t="b">
+      <c r="AH10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH10" t="s">
+      <c r="AI10" t="s">
         <v>94</v>
       </c>
-      <c r="AI10" t="s">
+      <c r="AJ10" t="s">
         <v>95</v>
       </c>
-      <c r="AJ10" s="3" t="s">
+      <c r="AK10" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AK10" s="3" t="s">
+      <c r="AL10" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AL10" t="s">
+      <c r="AM10" t="s">
         <v>97</v>
       </c>
-      <c r="AN10" t="s">
+      <c r="AO10" t="s">
         <v>98</v>
       </c>
-      <c r="AP10" t="s">
+      <c r="AQ10" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:43" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>1415</v>
       </c>
@@ -5335,50 +5411,50 @@
       <c r="X11" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="Y11" t="s">
+      <c r="Z11" t="s">
         <v>375</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AB11" t="s">
         <v>376</v>
       </c>
-      <c r="AB11" s="3" t="s">
+      <c r="AC11" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="AC11" s="8" t="s">
+      <c r="AD11" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD11" t="s">
+      <c r="AE11" t="s">
         <v>378</v>
       </c>
-      <c r="AF11" t="s">
+      <c r="AG11" t="s">
         <v>379</v>
       </c>
-      <c r="AG11" s="3" t="b">
+      <c r="AH11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH11" t="s">
+      <c r="AI11" t="s">
         <v>380</v>
       </c>
-      <c r="AI11" t="s">
+      <c r="AJ11" t="s">
         <v>381</v>
       </c>
-      <c r="AJ11" s="3" t="s">
+      <c r="AK11" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AK11" s="3" t="s">
+      <c r="AL11" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AL11" t="s">
+      <c r="AM11" t="s">
         <v>382</v>
       </c>
-      <c r="AN11" t="s">
+      <c r="AO11" t="s">
         <v>383</v>
       </c>
-      <c r="AP11" t="s">
+      <c r="AQ11" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>1678</v>
       </c>
@@ -5442,47 +5518,50 @@
       <c r="X12" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="Y12" t="s">
+      <c r="Y12" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="Z12" t="s">
         <v>437</v>
       </c>
-      <c r="AA12" t="s">
+      <c r="AB12" t="s">
         <v>438</v>
       </c>
-      <c r="AB12" s="3" t="s">
+      <c r="AC12" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AC12" s="8" t="s">
+      <c r="AD12" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD12" t="s">
+      <c r="AE12" t="s">
         <v>439</v>
       </c>
-      <c r="AE12" t="s">
+      <c r="AF12" t="s">
         <v>138</v>
       </c>
-      <c r="AG12" s="3" t="b">
+      <c r="AH12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH12" t="s">
+      <c r="AI12" t="s">
         <v>440</v>
       </c>
-      <c r="AI12" t="s">
+      <c r="AJ12" t="s">
         <v>441</v>
       </c>
-      <c r="AJ12" s="3" t="s">
+      <c r="AK12" s="3" t="s">
         <v>546</v>
       </c>
-      <c r="AK12" s="3" t="s">
+      <c r="AL12" s="3" t="s">
         <v>529</v>
       </c>
-      <c r="AL12" t="s">
+      <c r="AM12" t="s">
         <v>442</v>
       </c>
-      <c r="AM12" t="s">
+      <c r="AN12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>5078</v>
       </c>
@@ -5543,47 +5622,50 @@
       <c r="X13" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="Y13" t="s">
+      <c r="Y13" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="Z13" t="s">
         <v>59</v>
       </c>
-      <c r="AA13" t="s">
+      <c r="AB13" t="s">
         <v>60</v>
       </c>
-      <c r="AB13" s="3" t="s">
+      <c r="AC13" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="AC13" s="8" t="s">
+      <c r="AD13" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="AD13" t="s">
+      <c r="AE13" t="s">
         <v>63</v>
       </c>
-      <c r="AF13" t="s">
+      <c r="AG13" t="s">
         <v>64</v>
       </c>
-      <c r="AG13" s="3" t="b">
+      <c r="AH13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH13" t="s">
+      <c r="AI13" t="s">
         <v>65</v>
       </c>
-      <c r="AI13" t="s">
+      <c r="AJ13" t="s">
         <v>66</v>
       </c>
-      <c r="AJ13" s="3" t="s">
+      <c r="AK13" s="3" t="s">
         <v>547</v>
       </c>
-      <c r="AK13" s="3" t="s">
+      <c r="AL13" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AL13" t="s">
+      <c r="AM13" t="s">
         <v>69</v>
       </c>
-      <c r="AN13" t="s">
+      <c r="AO13" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>5171</v>
       </c>
@@ -5611,23 +5693,26 @@
       <c r="X14" s="3" t="s">
         <v>474</v>
       </c>
-      <c r="AB14" s="3" t="s">
+      <c r="Y14" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="AC14" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AG14" s="3" t="b">
+      <c r="AH14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AJ14" s="3" t="s">
+      <c r="AK14" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AK14" s="3" t="s">
+      <c r="AL14" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AO14" t="s">
+      <c r="AP14" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>5281</v>
       </c>
@@ -5691,48 +5776,51 @@
       <c r="X15" s="3" t="s">
         <v>552</v>
       </c>
-      <c r="Y15" t="s">
+      <c r="Y15" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="Z15" t="s">
         <v>310</v>
       </c>
-      <c r="Z15" t="s">
+      <c r="AA15" t="s">
         <v>138</v>
       </c>
-      <c r="AB15" s="3" t="s">
+      <c r="AC15" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="AC15" s="8" t="s">
+      <c r="AD15" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD15" t="s">
+      <c r="AE15" t="s">
         <v>311</v>
       </c>
-      <c r="AE15" t="s">
+      <c r="AF15" t="s">
         <v>117</v>
       </c>
-      <c r="AG15" s="3" t="b">
+      <c r="AH15" s="3" t="b">
         <v>1</v>
       </c>
-      <c r="AH15" t="s">
+      <c r="AI15" t="s">
         <v>312</v>
       </c>
-      <c r="AI15" t="s">
+      <c r="AJ15" t="s">
         <v>313</v>
       </c>
-      <c r="AJ15" s="3" t="s">
+      <c r="AK15" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="AK15" s="3" t="s">
+      <c r="AL15" s="3" t="s">
         <v>529</v>
       </c>
-      <c r="AL15" t="s">
+      <c r="AM15" t="s">
         <v>315</v>
       </c>
-      <c r="AN15" t="s">
+      <c r="AO15" t="s">
         <v>316</v>
       </c>
-      <c r="AP15" s="6"/>
+      <c r="AQ15" s="6"/>
     </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>6502</v>
       </c>
@@ -5796,50 +5884,53 @@
       <c r="X16" s="3" t="s">
         <v>552</v>
       </c>
-      <c r="Y16" t="s">
+      <c r="Y16" s="3" t="s">
+        <v>574</v>
+      </c>
+      <c r="Z16" t="s">
         <v>396</v>
       </c>
-      <c r="AA16" t="s">
+      <c r="AB16" t="s">
         <v>397</v>
       </c>
-      <c r="AB16" s="3" t="s">
+      <c r="AC16" s="3" t="s">
         <v>543</v>
       </c>
-      <c r="AC16" s="8" t="s">
+      <c r="AD16" s="8" t="s">
         <v>398</v>
       </c>
-      <c r="AD16" t="s">
+      <c r="AE16" t="s">
         <v>399</v>
       </c>
-      <c r="AF16" t="s">
+      <c r="AG16" t="s">
         <v>400</v>
       </c>
-      <c r="AG16" s="3" t="b">
+      <c r="AH16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH16" t="s">
+      <c r="AI16" t="s">
         <v>401</v>
       </c>
-      <c r="AI16" t="s">
+      <c r="AJ16" t="s">
         <v>402</v>
       </c>
-      <c r="AJ16" s="3" t="s">
+      <c r="AK16" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AK16" s="3" t="s">
+      <c r="AL16" s="3" t="s">
         <v>529</v>
       </c>
-      <c r="AL16" t="s">
+      <c r="AM16" t="s">
         <v>403</v>
       </c>
-      <c r="AM16" t="s">
+      <c r="AN16" t="s">
         <v>117</v>
       </c>
-      <c r="AP16" t="s">
+      <c r="AQ16" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="17" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>8058</v>
       </c>
@@ -5903,47 +5994,50 @@
       <c r="X17" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="Y17" t="s">
+      <c r="Y17" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="Z17" t="s">
         <v>267</v>
       </c>
-      <c r="AA17" t="s">
+      <c r="AB17" t="s">
         <v>268</v>
       </c>
-      <c r="AB17" s="3" t="s">
+      <c r="AC17" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="AC17" s="8" t="s">
+      <c r="AD17" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD17" t="s">
+      <c r="AE17" t="s">
         <v>269</v>
       </c>
-      <c r="AE17" t="s">
+      <c r="AF17" t="s">
         <v>117</v>
       </c>
-      <c r="AG17" s="3" t="b">
+      <c r="AH17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH17" t="s">
+      <c r="AI17" t="s">
         <v>270</v>
       </c>
-      <c r="AI17" t="s">
+      <c r="AJ17" t="s">
         <v>271</v>
       </c>
-      <c r="AJ17" s="3" t="s">
+      <c r="AK17" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="AK17" s="3" t="s">
+      <c r="AL17" s="3" t="s">
         <v>553</v>
       </c>
-      <c r="AL17" t="s">
+      <c r="AM17" t="s">
         <v>272</v>
       </c>
-      <c r="AN17" t="s">
+      <c r="AO17" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>10064</v>
       </c>
@@ -6007,47 +6101,50 @@
       <c r="X18" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Y18" t="s">
+      <c r="Y18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z18" t="s">
         <v>180</v>
       </c>
-      <c r="AA18" t="s">
+      <c r="AB18" t="s">
         <v>181</v>
       </c>
-      <c r="AB18" s="3" t="s">
+      <c r="AC18" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="AC18" s="8" t="s">
+      <c r="AD18" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="AD18" t="s">
+      <c r="AE18" t="s">
         <v>184</v>
       </c>
-      <c r="AF18" t="s">
+      <c r="AG18" t="s">
         <v>185</v>
       </c>
-      <c r="AG18" s="3" t="b">
+      <c r="AH18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH18" t="s">
+      <c r="AI18" t="s">
         <v>186</v>
       </c>
-      <c r="AI18" t="s">
+      <c r="AJ18" t="s">
         <v>187</v>
       </c>
-      <c r="AJ18" s="3" t="s">
+      <c r="AK18" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="AK18" s="3" t="s">
+      <c r="AL18" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="AL18" t="s">
+      <c r="AM18" t="s">
         <v>189</v>
       </c>
-      <c r="AN18" t="s">
+      <c r="AO18" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:43" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>13648</v>
       </c>
@@ -6111,50 +6208,50 @@
       <c r="X19" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Y19" t="s">
+      <c r="Z19" t="s">
         <v>519</v>
       </c>
-      <c r="Z19" t="s">
+      <c r="AA19" t="s">
         <v>520</v>
       </c>
-      <c r="AB19" s="3" t="s">
+      <c r="AC19" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="AC19" s="8" t="s">
+      <c r="AD19" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD19" t="s">
+      <c r="AE19" t="s">
         <v>521</v>
       </c>
-      <c r="AE19" t="s">
+      <c r="AF19" t="s">
         <v>138</v>
       </c>
-      <c r="AG19" s="3" t="b">
+      <c r="AH19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH19" t="s">
+      <c r="AI19" t="s">
         <v>522</v>
       </c>
-      <c r="AI19" t="s">
+      <c r="AJ19" t="s">
         <v>523</v>
-      </c>
-      <c r="AJ19" s="3" t="s">
-        <v>88</v>
       </c>
       <c r="AK19" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AL19" t="s">
+      <c r="AL19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="AM19" t="s">
         <v>524</v>
       </c>
-      <c r="AM19" t="s">
+      <c r="AN19" t="s">
         <v>138</v>
       </c>
-      <c r="AP19" t="s">
+      <c r="AQ19" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:43" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>120956</v>
       </c>
@@ -6218,50 +6315,50 @@
       <c r="X20" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Y20" t="s">
+      <c r="Z20" t="s">
         <v>287</v>
       </c>
-      <c r="AA20" t="s">
+      <c r="AB20" t="s">
         <v>288</v>
       </c>
-      <c r="AB20" s="3" t="s">
+      <c r="AC20" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="AC20" s="8" t="s">
+      <c r="AD20" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="AD20" t="s">
+      <c r="AE20" t="s">
         <v>291</v>
       </c>
-      <c r="AF20" t="s">
+      <c r="AG20" t="s">
         <v>292</v>
       </c>
-      <c r="AG20" s="3" t="b">
+      <c r="AH20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH20" t="s">
+      <c r="AI20" t="s">
         <v>293</v>
       </c>
-      <c r="AI20" t="s">
+      <c r="AJ20" t="s">
         <v>294</v>
       </c>
-      <c r="AJ20" s="3" t="s">
+      <c r="AK20" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AK20" s="3" t="s">
+      <c r="AL20" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="AL20" t="s">
+      <c r="AM20" t="s">
         <v>295</v>
       </c>
-      <c r="AN20" t="s">
+      <c r="AO20" t="s">
         <v>296</v>
       </c>
-      <c r="AP20" t="s">
+      <c r="AQ20" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>232677</v>
       </c>
@@ -6325,47 +6422,50 @@
       <c r="X21" s="3" t="s">
         <v>474</v>
       </c>
-      <c r="Y21" t="s">
+      <c r="Y21" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="Z21" t="s">
         <v>113</v>
       </c>
-      <c r="AA21" t="s">
+      <c r="AB21" t="s">
         <v>114</v>
       </c>
-      <c r="AB21" s="3" t="s">
+      <c r="AC21" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="AC21" s="8" t="s">
+      <c r="AD21" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD21" t="s">
+      <c r="AE21" t="s">
         <v>116</v>
       </c>
-      <c r="AE21" t="s">
+      <c r="AF21" t="s">
         <v>117</v>
       </c>
-      <c r="AG21" s="3" t="b">
+      <c r="AH21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH21" t="s">
+      <c r="AI21" t="s">
         <v>118</v>
       </c>
-      <c r="AI21" t="s">
+      <c r="AJ21" t="s">
         <v>119</v>
       </c>
-      <c r="AJ21" s="3" t="s">
+      <c r="AK21" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AK21" s="3" t="s">
+      <c r="AL21" s="3" t="s">
         <v>529</v>
       </c>
-      <c r="AL21" t="s">
+      <c r="AM21" t="s">
         <v>120</v>
       </c>
-      <c r="AN21" t="s">
+      <c r="AO21" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>244602</v>
       </c>
@@ -6429,47 +6529,50 @@
       <c r="X22" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="Y22" t="s">
+      <c r="Y22" s="3" t="s">
+        <v>577</v>
+      </c>
+      <c r="Z22" t="s">
         <v>455</v>
       </c>
-      <c r="AA22" t="s">
+      <c r="AB22" t="s">
         <v>456</v>
       </c>
-      <c r="AB22" s="3" t="s">
+      <c r="AC22" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AC22" s="8" t="s">
+      <c r="AD22" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD22" t="s">
+      <c r="AE22" t="s">
         <v>457</v>
       </c>
-      <c r="AE22" t="s">
+      <c r="AF22" t="s">
         <v>117</v>
       </c>
-      <c r="AG22" s="3" t="b">
+      <c r="AH22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH22" t="s">
+      <c r="AI22" t="s">
         <v>458</v>
       </c>
-      <c r="AI22" t="s">
+      <c r="AJ22" t="s">
         <v>459</v>
       </c>
-      <c r="AJ22" s="3" t="s">
+      <c r="AK22" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AK22" s="3" t="s">
+      <c r="AL22" s="3" t="s">
         <v>529</v>
       </c>
-      <c r="AL22" t="s">
+      <c r="AM22" t="s">
         <v>460</v>
       </c>
-      <c r="AN22" t="s">
+      <c r="AO22" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>249273</v>
       </c>
@@ -6531,49 +6634,52 @@
         <v>266</v>
       </c>
       <c r="X23" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="Y23" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Y23" t="s">
+      <c r="Z23" t="s">
         <v>496</v>
       </c>
-      <c r="AA23" t="s">
+      <c r="AB23" t="s">
         <v>497</v>
       </c>
-      <c r="AB23" s="3" t="s">
+      <c r="AC23" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AC23" s="8" t="s">
+      <c r="AD23" s="8" t="s">
         <v>498</v>
       </c>
-      <c r="AD23" t="s">
+      <c r="AE23" t="s">
         <v>499</v>
       </c>
-      <c r="AF23" t="s">
+      <c r="AG23" t="s">
         <v>500</v>
       </c>
-      <c r="AG23" s="3" t="b">
+      <c r="AH23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH23" t="s">
+      <c r="AI23" t="s">
         <v>501</v>
       </c>
-      <c r="AI23" t="s">
+      <c r="AJ23" t="s">
         <v>502</v>
       </c>
-      <c r="AJ23" s="3" t="s">
+      <c r="AK23" s="3" t="s">
         <v>503</v>
       </c>
-      <c r="AK23" s="3" t="s">
+      <c r="AL23" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AL23" t="s">
+      <c r="AM23" t="s">
         <v>504</v>
       </c>
-      <c r="AN23" t="s">
+      <c r="AO23" t="s">
         <v>505</v>
       </c>
     </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>250635</v>
       </c>
@@ -6637,47 +6743,50 @@
       <c r="X24" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="Y24" t="s">
+      <c r="Y24" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="Z24" t="s">
         <v>201</v>
       </c>
-      <c r="AA24" t="s">
+      <c r="AB24" t="s">
         <v>203</v>
       </c>
-      <c r="AB24" s="3" t="s">
+      <c r="AC24" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="AC24" s="8" t="s">
+      <c r="AD24" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD24" t="s">
+      <c r="AE24" t="s">
         <v>204</v>
       </c>
-      <c r="AE24" t="s">
+      <c r="AF24" t="s">
         <v>138</v>
       </c>
-      <c r="AG24" s="3" t="b">
+      <c r="AH24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH24" t="s">
+      <c r="AI24" t="s">
         <v>205</v>
       </c>
-      <c r="AI24" t="s">
+      <c r="AJ24" t="s">
         <v>206</v>
       </c>
-      <c r="AJ24" s="3" t="s">
+      <c r="AK24" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="AK24" s="3" t="s">
+      <c r="AL24" s="3" t="s">
         <v>553</v>
       </c>
-      <c r="AL24" t="s">
+      <c r="AM24" t="s">
         <v>208</v>
       </c>
-      <c r="AN24" t="s">
+      <c r="AO24" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:43" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>259944</v>
       </c>
@@ -6741,47 +6850,57 @@
       <c r="X25" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="Y25" t="s">
+      <c r="Y25" s="3" t="s">
+        <v>578</v>
+      </c>
+      <c r="Z25" t="s">
         <v>158</v>
       </c>
-      <c r="AA25" t="s">
+      <c r="AB25" t="s">
         <v>159</v>
       </c>
-      <c r="AB25" s="3" t="s">
+      <c r="AC25" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="AC25" s="8" t="s">
+      <c r="AD25" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="AD25" t="s">
+      <c r="AE25" t="s">
         <v>160</v>
       </c>
-      <c r="AE25" t="s">
+      <c r="AF25" t="s">
         <v>138</v>
       </c>
-      <c r="AG25" s="3" t="b">
+      <c r="AH25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="AH25" t="s">
+      <c r="AI25" t="s">
         <v>161</v>
       </c>
-      <c r="AI25" t="s">
+      <c r="AJ25" t="s">
         <v>162</v>
       </c>
-      <c r="AJ25" s="3" t="s">
+      <c r="AK25" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AK25" s="3" t="s">
+      <c r="AL25" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="AL25" t="s">
+      <c r="AM25" t="s">
         <v>165</v>
       </c>
-      <c r="AN25" t="s">
+      <c r="AO25" t="s">
         <v>166</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AQ25">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="VRAI"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState ref="A2:AO25">
     <sortCondition ref="A2:A25"/>
   </sortState>

</xml_diff>